<commit_message>
due to a push error
</commit_message>
<xml_diff>
--- a/lai/valuationquan/szseinnovation100index/szseinnovation100indexmodel1prac.xlsx
+++ b/lai/valuationquan/szseinnovation100index/szseinnovation100indexmodel1prac.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="975">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="956">
   <si>
     <t>PE</t>
   </si>
@@ -3831,82 +3831,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026/3/27
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/1
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/2
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/3
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/7
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/8
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/9
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/10
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/13
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/14
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/15
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/16
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/17
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/20
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/21
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/22
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/24
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/27
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/28
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026/4/23
 </t>
   </si>
 </sst>
@@ -5943,11 +5867,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="588371840"/>
-        <c:axId val="588378496"/>
+        <c:axId val="393928064"/>
+        <c:axId val="395000832"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="588371840"/>
+        <c:axId val="393928064"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5990,14 +5914,14 @@
             <a:endParaRPr lang="zh-CN"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="588378496"/>
+        <c:crossAx val="395000832"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
         <c:baseTimeUnit val="days"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="588378496"/>
+        <c:axId val="395000832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6048,7 +5972,7 @@
             <a:endParaRPr lang="zh-CN"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="588371840"/>
+        <c:crossAx val="393928064"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9016,7 +8940,7 @@
   <sheetPr codeName="Sheet4">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D1230"/>
+  <dimension ref="A1:D1210"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="9" style="18"/>
@@ -27107,7 +27031,7 @@
     </row>
     <row r="1132" spans="1:4">
       <c r="A1132" s="18">
-        <f t="shared" ref="A1132:A1226" si="7">A1131+1</f>
+        <f t="shared" ref="A1132:A1210" si="7">A1131+1</f>
         <v>1130</v>
       </c>
       <c r="B1132" s="30">
@@ -28367,326 +28291,6 @@
       <c r="D1210" s="18">
         <f>SUM(C$3:C1210)/A1210</f>
         <v>26.136981933917117</v>
-      </c>
-    </row>
-    <row r="1211" spans="1:4">
-      <c r="A1211" s="18">
-        <f t="shared" si="7"/>
-        <v>1209</v>
-      </c>
-      <c r="B1211" s="30" t="s">
-        <v>956</v>
-      </c>
-      <c r="C1211" s="31">
-        <v>30.549999239999998</v>
-      </c>
-      <c r="D1211" s="18">
-        <f>SUM(C$3:C1211)/A1211</f>
-        <v>26.140632072300974</v>
-      </c>
-    </row>
-    <row r="1212" spans="1:4">
-      <c r="A1212" s="18">
-        <f t="shared" si="7"/>
-        <v>1210</v>
-      </c>
-      <c r="B1212" s="30" t="s">
-        <v>957</v>
-      </c>
-      <c r="C1212" s="31">
-        <v>30.340000150000002</v>
-      </c>
-      <c r="D1212" s="18">
-        <f>SUM(C$3:C1212)/A1212</f>
-        <v>26.144102624431305</v>
-      </c>
-    </row>
-    <row r="1213" spans="1:4">
-      <c r="A1213" s="18">
-        <f t="shared" si="7"/>
-        <v>1211</v>
-      </c>
-      <c r="B1213" s="30" t="s">
-        <v>958</v>
-      </c>
-      <c r="C1213" s="31">
-        <v>29.940000529999999</v>
-      </c>
-      <c r="D1213" s="18">
-        <f>SUM(C$3:C1213)/A1213</f>
-        <v>26.147237139629958</v>
-      </c>
-    </row>
-    <row r="1214" spans="1:4">
-      <c r="A1214" s="18">
-        <f t="shared" si="7"/>
-        <v>1212</v>
-      </c>
-      <c r="B1214" s="30" t="s">
-        <v>959</v>
-      </c>
-      <c r="C1214" s="31">
-        <v>29.979999540000001</v>
-      </c>
-      <c r="D1214" s="18">
-        <f>SUM(C$3:C1214)/A1214</f>
-        <v>26.150399484844783</v>
-      </c>
-    </row>
-    <row r="1215" spans="1:4">
-      <c r="A1215" s="18">
-        <f t="shared" si="7"/>
-        <v>1213</v>
-      </c>
-      <c r="B1215" s="30" t="s">
-        <v>960</v>
-      </c>
-      <c r="C1215" s="31">
-        <v>31.379999160000001</v>
-      </c>
-      <c r="D1215" s="18">
-        <f>SUM(C$3:C1215)/A1215</f>
-        <v>26.154710778888603</v>
-      </c>
-    </row>
-    <row r="1216" spans="1:4">
-      <c r="A1216" s="18">
-        <f t="shared" si="7"/>
-        <v>1214</v>
-      </c>
-      <c r="B1216" s="30" t="s">
-        <v>961</v>
-      </c>
-      <c r="C1216" s="31">
-        <v>31.299999239999998</v>
-      </c>
-      <c r="D1216" s="18">
-        <f>SUM(C$3:C1216)/A1216</f>
-        <v>26.158949072513902</v>
-      </c>
-    </row>
-    <row r="1217" spans="1:4">
-      <c r="A1217" s="18">
-        <f t="shared" si="7"/>
-        <v>1215</v>
-      </c>
-      <c r="B1217" s="30" t="s">
-        <v>962</v>
-      </c>
-      <c r="C1217" s="31">
-        <v>32.38999939</v>
-      </c>
-      <c r="D1217" s="18">
-        <f>SUM(C$3:C1217)/A1217</f>
-        <v>26.164077508989202</v>
-      </c>
-    </row>
-    <row r="1218" spans="1:4">
-      <c r="A1218" s="18">
-        <f t="shared" si="7"/>
-        <v>1216</v>
-      </c>
-      <c r="B1218" s="30" t="s">
-        <v>963</v>
-      </c>
-      <c r="C1218" s="31">
-        <v>32.72000122</v>
-      </c>
-      <c r="D1218" s="18">
-        <f>SUM(C$3:C1218)/A1218</f>
-        <v>26.169468893619968</v>
-      </c>
-    </row>
-    <row r="1219" spans="1:4">
-      <c r="A1219" s="18">
-        <f t="shared" si="7"/>
-        <v>1217</v>
-      </c>
-      <c r="B1219" s="30" t="s">
-        <v>964</v>
-      </c>
-      <c r="C1219" s="31">
-        <v>33.349998470000003</v>
-      </c>
-      <c r="D1219" s="18">
-        <f>SUM(C$3:C1219)/A1219</f>
-        <v>26.175369082261199</v>
-      </c>
-    </row>
-    <row r="1220" spans="1:4">
-      <c r="A1220" s="18">
-        <f t="shared" si="7"/>
-        <v>1218</v>
-      </c>
-      <c r="B1220" s="30" t="s">
-        <v>965</v>
-      </c>
-      <c r="C1220" s="31">
-        <v>33.060001370000002</v>
-      </c>
-      <c r="D1220" s="18">
-        <f>SUM(C$3:C1220)/A1220</f>
-        <v>26.181021489722394</v>
-      </c>
-    </row>
-    <row r="1221" spans="1:4">
-      <c r="A1221" s="18">
-        <f t="shared" si="7"/>
-        <v>1219</v>
-      </c>
-      <c r="B1221" s="30" t="s">
-        <v>966</v>
-      </c>
-      <c r="C1221" s="31">
-        <v>33.799999239999998</v>
-      </c>
-      <c r="D1221" s="18">
-        <f>SUM(C$3:C1221)/A1221</f>
-        <v>26.187271676556094</v>
-      </c>
-    </row>
-    <row r="1222" spans="1:4">
-      <c r="A1222" s="18">
-        <f t="shared" si="7"/>
-        <v>1220</v>
-      </c>
-      <c r="B1222" s="30" t="s">
-        <v>967</v>
-      </c>
-      <c r="C1222" s="31">
-        <v>33.91999817</v>
-      </c>
-      <c r="D1222" s="18">
-        <f>SUM(C$3:C1222)/A1222</f>
-        <v>26.193609976960555</v>
-      </c>
-    </row>
-    <row r="1223" spans="1:4">
-      <c r="A1223" s="18">
-        <f t="shared" si="7"/>
-        <v>1221</v>
-      </c>
-      <c r="B1223" s="30" t="s">
-        <v>968</v>
-      </c>
-      <c r="C1223" s="31">
-        <v>34.040000919999997</v>
-      </c>
-      <c r="D1223" s="18">
-        <f>SUM(C$3:C1223)/A1223</f>
-        <v>26.200036177569103</v>
-      </c>
-    </row>
-    <row r="1224" spans="1:4">
-      <c r="A1224" s="18">
-        <f t="shared" si="7"/>
-        <v>1222</v>
-      </c>
-      <c r="B1224" s="30" t="s">
-        <v>969</v>
-      </c>
-      <c r="C1224" s="31">
-        <v>34.159999849999998</v>
-      </c>
-      <c r="D1224" s="18">
-        <f>SUM(C$3:C1224)/A1224</f>
-        <v>26.206550059461435</v>
-      </c>
-    </row>
-    <row r="1225" spans="1:4">
-      <c r="A1225" s="18">
-        <f t="shared" si="7"/>
-        <v>1223</v>
-      </c>
-      <c r="B1225" s="30" t="s">
-        <v>970</v>
-      </c>
-      <c r="C1225" s="31">
-        <v>34.380001069999999</v>
-      </c>
-      <c r="D1225" s="18">
-        <f>SUM(C$3:C1225)/A1225</f>
-        <v>26.213233175577983</v>
-      </c>
-    </row>
-    <row r="1226" spans="1:4">
-      <c r="A1226" s="18">
-        <f t="shared" si="7"/>
-        <v>1224</v>
-      </c>
-      <c r="B1226" s="30" t="s">
-        <v>974</v>
-      </c>
-      <c r="C1226" s="31">
-        <v>34.32</v>
-      </c>
-      <c r="D1226" s="18">
-        <f>SUM(C$3:C1226)/A1226</f>
-        <v>26.219856351088133</v>
-      </c>
-    </row>
-    <row r="1227" spans="1:4">
-      <c r="A1227" s="18">
-        <f t="shared" ref="A1227:A1230" si="8">A1226+1</f>
-        <v>1225</v>
-      </c>
-      <c r="B1227" s="30" t="s">
-        <v>971</v>
-      </c>
-      <c r="C1227" s="31">
-        <v>34.25</v>
-      </c>
-      <c r="D1227" s="18">
-        <f>SUM(C$3:C1227)/A1227</f>
-        <v>26.226411570393367</v>
-      </c>
-    </row>
-    <row r="1228" spans="1:4">
-      <c r="A1228" s="18">
-        <f t="shared" si="8"/>
-        <v>1226</v>
-      </c>
-      <c r="B1228" s="30" t="s">
-        <v>972</v>
-      </c>
-      <c r="C1228" s="31">
-        <v>34.270000459999999</v>
-      </c>
-      <c r="D1228" s="18">
-        <f>SUM(C$3:C1228)/A1228</f>
-        <v>26.232972409618167</v>
-      </c>
-    </row>
-    <row r="1229" spans="1:4">
-      <c r="A1229" s="18">
-        <f t="shared" si="8"/>
-        <v>1227</v>
-      </c>
-      <c r="B1229" s="30" t="s">
-        <v>973</v>
-      </c>
-      <c r="C1229" s="31">
-        <v>33.75</v>
-      </c>
-      <c r="D1229" s="18">
-        <f>SUM(C$3:C1229)/A1229</f>
-        <v>26.239098756472597</v>
-      </c>
-    </row>
-    <row r="1230" spans="1:4">
-      <c r="A1230" s="18">
-        <f t="shared" si="8"/>
-        <v>1228</v>
-      </c>
-      <c r="B1230" s="30">
-        <v>46141</v>
-      </c>
-      <c r="C1230" s="31">
-        <v>34.459999080000003</v>
-      </c>
-      <c r="D1230" s="18">
-        <f>SUM(C$3:C1230)/A1230</f>
-        <v>26.245793300709998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>